<commit_message>
corrected paths in R scripts
</commit_message>
<xml_diff>
--- a/Supplementary_Materials/Supplementary_tables.xlsx
+++ b/Supplementary_Materials/Supplementary_tables.xlsx
@@ -17,11 +17,11 @@
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1752044485" val="1050" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1752044485" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1752044485" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1752044485"/>
-      <pm:sortOptions xmlns:pm="smNativeData" id="1752044485" headings="1">
+      <pm:revision xmlns:pm="smNativeData" day="1752046170" val="1050" rev="124" rev64="64" revOS="3" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1752046170" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1752046170" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1752046170"/>
+      <pm:sortOptions xmlns:pm="smNativeData" id="1752046170" headings="1">
         <pm:column colId="1" sortType="descending"/>
         <pm:column colId="2"/>
         <pm:column colId="-1"/>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2067" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2073" uniqueCount="742">
   <si>
     <t>Table S1. Coordinates of sampling points (supporting information for Fig. 2)</t>
   </si>
@@ -1707,6 +1707,9 @@
   </si>
   <si>
     <t>Depth</t>
+  </si>
+  <si>
+    <t>Sample</t>
   </si>
   <si>
     <t>#</t>
@@ -2344,7 +2347,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -2359,7 +2362,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Basic Sans" sz="200" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -2376,7 +2379,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default" weight="bold" i="1"/>
             <pm:cs face="Basic Roman" sz="200" lang="default" weight="bold" i="1"/>
             <pm:ea face="Basic Roman" sz="200" lang="default" weight="bold" i="1"/>
@@ -2392,7 +2395,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default" i="1"/>
             <pm:cs face="Basic Roman" sz="200" lang="default" i="1"/>
             <pm:ea face="Basic Roman" sz="200" lang="default" i="1"/>
@@ -2407,7 +2410,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="220" lang="default"/>
             <pm:ea face="Basic Roman" sz="220" lang="default"/>
@@ -2423,7 +2426,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="200" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="200" lang="default" weight="bold"/>
@@ -2440,7 +2443,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" fgClr="222222" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" fgClr="222222" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="220" lang="default" weight="bold" i="1"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold" i="1"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold" i="1"/>
@@ -2456,7 +2459,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="220" lang="default" i="1"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" i="1"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" i="1"/>
@@ -2473,7 +2476,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="220" lang="default" weight="bold" i="1"/>
             <pm:cs face="Basic Roman" sz="220" lang="default" weight="bold" i="1"/>
             <pm:ea face="Basic Roman" sz="220" lang="default" weight="bold" i="1"/>
@@ -2488,7 +2491,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="220" lang="default"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -2504,7 +2507,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default" weight="bold"/>
             <pm:cs face="Basic Roman" sz="200" lang="default" weight="bold"/>
             <pm:ea face="Basic Roman" sz="200" lang="default" weight="bold"/>
@@ -2520,7 +2523,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1752044485" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1752046170" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="220" lang="default" i="1"/>
             <pm:cs face="Basic Roman" sz="200" lang="default"/>
             <pm:ea face="Basic Roman" sz="200" lang="default"/>
@@ -2529,7 +2532,7 @@
       </extLst>
     </font>
   </fonts>
-  <fills count="43">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2545,7 +2548,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="004A86E8" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="004A86E8" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2556,7 +2559,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="004A86E8" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="004A86E8" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2570,7 +2573,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="004A86E8" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="004A86E8" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2581,7 +2584,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="004285F4" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="004285F4" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2592,7 +2595,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00D8E5F8" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00D8E5F8" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2615,7 +2618,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00833C0C" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00833C0C" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2626,7 +2629,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00C65911" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00C65911" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2637,7 +2640,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00F4AF82" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00F4AF82" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2648,7 +2651,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00F8CAAB" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00F8CAAB" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2659,7 +2662,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00FEF5F0" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00FEF5F0" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2670,7 +2673,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00203764" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00203764" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2681,7 +2684,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00305496" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00305496" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2692,7 +2695,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="008EA9DB" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="008EA9DB" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2703,7 +2706,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00D9E1F2" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00D9E1F2" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2714,7 +2717,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2725,7 +2728,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2736,7 +2739,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2747,7 +2750,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00FDE9D9" bgLvl="0" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2758,7 +2761,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="12" fgClr="007F7F00" bgLvl="88" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="12" fgClr="007F7F00" bgLvl="88" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2769,7 +2772,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="12" fgClr="00FF0000" bgLvl="88" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="12" fgClr="00FF0000" bgLvl="88" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2780,7 +2783,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="12" fgClr="00FF0000" bgLvl="88" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="12" fgClr="00FF0000" bgLvl="88" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2791,7 +2794,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="12" fgClr="00FF0000" bgLvl="88" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="12" fgClr="00FF0000" bgLvl="88" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2802,7 +2805,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="12" fgClr="007F7F00" bgLvl="88" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="12" fgClr="007F7F00" bgLvl="88" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2813,7 +2816,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="12" fgClr="00FFFF00" bgLvl="88" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="12" fgClr="00FFFF00" bgLvl="88" bgClr="00FFFFFF"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2824,7 +2827,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="85" fgClr="00FFFFFF" bgLvl="15" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -2835,112 +2838,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF010180"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="50" fgClr="000000FF" bgLvl="50" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0000A3"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="64" fgClr="000000FF" bgLvl="36" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD100D1"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="82" fgClr="00FF00FF" bgLvl="18" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF00FF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00FF00FF" bgLvl="0" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF3DFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="76" fgClr="00FF00FF" bgLvl="24" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF5CFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="64" fgClr="00FF00FF" bgLvl="36" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCECE9E"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="38" fgClr="007F7F00" bgLvl="62" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF333333"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="00333333" bgLvl="0" bgClr="00FFFFFF"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4D4D4D"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1752044485" type="1" fgLvl="100" fgClr="004D4D4D" bgLvl="0" bgClr="00FFFFFF"/>
+            <pm:shade xmlns:pm="smNativeData" id="1752046170" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="33">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -2956,7 +2860,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -2975,7 +2879,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -2996,7 +2900,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3015,7 +2919,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3036,7 +2940,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3057,7 +2961,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3078,7 +2982,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3097,7 +3001,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3116,7 +3020,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -3138,7 +3042,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3159,7 +3063,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -3181,7 +3085,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -3203,7 +3107,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3222,7 +3126,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3241,7 +3145,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3260,7 +3164,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3279,7 +3183,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3298,7 +3202,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3317,7 +3221,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3336,7 +3240,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3355,7 +3259,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3374,7 +3278,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3393,7 +3297,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3412,7 +3316,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3433,7 +3337,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3454,7 +3358,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3475,7 +3379,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -3497,7 +3401,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -3518,7 +3422,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485">
+          <pm:border xmlns:pm="smNativeData" id="1752046170">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -3540,7 +3444,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3559,7 +3463,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3578,7 +3482,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3597,178 +3501,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1752044485"/>
+          <pm:border xmlns:pm="smNativeData" id="1752046170"/>
         </ext>
       </extLst>
     </border>
@@ -3911,10 +3644,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1752044485" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1752046170" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1752044485" count="46">
+      <pm:colors xmlns:pm="smNativeData" id="1752046170" count="50">
         <pm:color name="Color 24" rgb="222222"/>
         <pm:color name="Color 25" rgb="4A86E8"/>
         <pm:color name="Color 26" rgb="4285F4"/>
@@ -3961,6 +3694,10 @@
         <pm:color name="Color 67" rgb="9E9E3D"/>
         <pm:color name="Color 68" rgb="ADAD5C"/>
         <pm:color name="Color 69" rgb="CECE9E"/>
+        <pm:color name="Color 70" rgb="0000A3"/>
+        <pm:color name="Color 71" rgb="D100D1"/>
+        <pm:color name="Color 72" rgb="FF3DFF"/>
+        <pm:color name="Color 73" rgb="FF5CFF"/>
       </pm:colors>
     </ext>
   </extLst>
@@ -4773,7 +4510,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1752044485" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1752046170" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4782,14 +4519,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752044485" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752046170" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5074,7 +4811,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1752044485" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1752046170" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5083,14 +4820,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752044485" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752046170" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -11150,7 +10887,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="127" spans="1:34" s="50" customFormat="1" ht="14.40" customHeight="1">
+    <row r="127" spans="1:33" s="50" customFormat="1" ht="14.40" customHeight="1">
       <c r="A127" s="43"/>
       <c r="B127" s="44"/>
       <c r="C127" s="44"/>
@@ -12458,7 +12195,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1752044485" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1752046170" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -12467,14 +12204,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752044485" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752046170" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -12546,55 +12283,55 @@
         <v>537</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>4</v>
+        <v>538</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="G3" s="21" t="s">
         <v>80</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="L3" s="40" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="M3" s="39" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="N3" s="39" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="O3" s="39" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="P3" s="40" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="R3" s="18" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="S3" s="18" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="T3" s="18" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="15.75" customHeight="1">
@@ -12602,7 +12339,7 @@
         <v>1000</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C4" s="26" t="n">
         <v>1</v>
@@ -12638,13 +12375,13 @@
         <v>0</v>
       </c>
       <c r="N4" s="26" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="O4" s="26" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="R4" s="28" t="n">
         <v>17.0941333770750994</v>
@@ -12662,7 +12399,7 @@
         <v>1000</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>9</v>
@@ -12723,7 +12460,7 @@
         <v>1000</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>17</v>
@@ -12784,7 +12521,7 @@
         <v>1000</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>25</v>
@@ -12833,7 +12570,7 @@
         <v>20.90962600708</v>
       </c>
       <c r="S7" s="28" t="n">
-        <v>14.474463462829501</v>
+        <v>14.4744634628294992</v>
       </c>
       <c r="T7" s="38">
         <f>S7-R7</f>
@@ -12845,7 +12582,7 @@
         <v>1000</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>33</v>
@@ -12906,7 +12643,7 @@
         <v>1000</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>34</v>
@@ -12952,7 +12689,7 @@
         <v>5.67109040074556958</v>
       </c>
       <c r="R9" s="28" t="n">
-        <v>21.256914138793892</v>
+        <v>21.2569141387938885</v>
       </c>
       <c r="S9" s="28" t="n">
         <v>15.9471893310545987</v>
@@ -12967,7 +12704,7 @@
         <v>1000</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>41</v>
@@ -13028,7 +12765,7 @@
         <v>650</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>2</v>
@@ -13074,7 +12811,7 @@
         <v>2.9635215946843898</v>
       </c>
       <c r="R11" s="28" t="n">
-        <v>23.5111398696898917</v>
+        <v>23.5111398696898881</v>
       </c>
       <c r="S11" s="28" t="n">
         <v>18.667835235595696</v>
@@ -13089,7 +12826,7 @@
         <v>650</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C12" s="26" t="n">
         <v>10</v>
@@ -13150,7 +12887,7 @@
         <v>650</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>18</v>
@@ -13211,7 +12948,7 @@
         <v>650</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C14" s="26" t="n">
         <v>26</v>
@@ -13260,7 +12997,7 @@
         <v>19.0198459625243999</v>
       </c>
       <c r="S14" s="28" t="n">
-        <v>15.3370389938353977</v>
+        <v>15.3370389938353959</v>
       </c>
       <c r="T14" s="38">
         <f>S14-R14</f>
@@ -13272,7 +13009,7 @@
         <v>650</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>31</v>
@@ -13321,19 +13058,19 @@
         <v>18.8960170745849005</v>
       </c>
       <c r="S15" s="28" t="n">
-        <v>13.8960628509520987</v>
+        <v>13.8960628509520969</v>
       </c>
       <c r="T15" s="38">
         <f>S15-R15</f>
         <v>-4.99995422363280007</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15.75" customHeight="1">
+    <row r="16" spans="1:20" ht="15.75" customHeight="1">
       <c r="A16" s="29" t="n">
         <v>650</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C16" s="26" t="n">
         <v>42</v>
@@ -13378,13 +13115,22 @@
         <f>4*O16*L16/D16</f>
         <v>30.0286813186813006</v>
       </c>
+      <c r="R16" t="s">
+        <v>555</v>
+      </c>
+      <c r="S16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T16" t="s">
+        <v>555</v>
+      </c>
     </row>
     <row r="17" spans="1:20" ht="15.75" customHeight="1">
       <c r="A17" s="30" t="n">
         <v>250</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C17" s="26" t="n">
         <v>3</v>
@@ -13445,7 +13191,7 @@
         <v>250</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C18" s="26" t="n">
         <v>11</v>
@@ -13506,7 +13252,7 @@
         <v>250</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C19" s="26" t="n">
         <v>19</v>
@@ -13567,7 +13313,7 @@
         <v>250</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C20" s="26" t="n">
         <v>27</v>
@@ -13613,7 +13359,7 @@
         <v>103.298453038673998</v>
       </c>
       <c r="R20" s="28" t="n">
-        <v>21.2792224884032919</v>
+        <v>21.2792224884032883</v>
       </c>
       <c r="S20" s="28" t="n">
         <v>16.1883792877196981</v>
@@ -13628,7 +13374,7 @@
         <v>250</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C21" s="26" t="n">
         <v>43</v>
@@ -13689,7 +13435,7 @@
         <v>100</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C22" s="26" t="n">
         <v>4</v>
@@ -13750,7 +13496,7 @@
         <v>100</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C23" s="26" t="n">
         <v>12</v>
@@ -13799,7 +13545,7 @@
         <v>14.2533750534056995</v>
       </c>
       <c r="S23" s="28" t="n">
-        <v>13.8370294570922017</v>
+        <v>13.8370294570921999</v>
       </c>
       <c r="T23" s="38">
         <f>S23-R23</f>
@@ -13811,7 +13557,7 @@
         <v>100</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C24" s="26" t="n">
         <v>20</v>
@@ -13857,10 +13603,10 @@
         <v>49.8022393425782965</v>
       </c>
       <c r="R24" s="28" t="n">
-        <v>19.8677425384520916</v>
+        <v>19.867742538452088</v>
       </c>
       <c r="S24" s="28" t="n">
-        <v>14.2873783111572017</v>
+        <v>14.2873783111571999</v>
       </c>
       <c r="T24" s="38">
         <f>S24-R24</f>
@@ -13872,7 +13618,7 @@
         <v>100</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C25" s="26" t="n">
         <v>28</v>
@@ -13933,7 +13679,7 @@
         <v>100</v>
       </c>
       <c r="B26" s="25" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C26" s="26" t="n">
         <v>44</v>
@@ -13989,12 +13735,12 @@
         <v>-3.59984207153320002</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="15.75" customHeight="1">
+    <row r="27" spans="1:20" ht="15.75" customHeight="1">
       <c r="A27" s="32" t="n">
         <v>25</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C27" s="26" t="n">
         <v>5</v>
@@ -14039,13 +13785,22 @@
         <f>4*O27*L27/D27</f>
         <v>19.3763231197772008</v>
       </c>
+      <c r="R27" t="s">
+        <v>555</v>
+      </c>
+      <c r="S27" t="s">
+        <v>555</v>
+      </c>
+      <c r="T27" t="s">
+        <v>555</v>
+      </c>
     </row>
     <row r="28" spans="1:20" ht="15.75" customHeight="1">
       <c r="A28" s="32" t="n">
         <v>25</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C28" s="26" t="n">
         <v>13</v>
@@ -14106,7 +13861,7 @@
         <v>25</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C29" s="26" t="n">
         <v>21</v>
@@ -14167,7 +13922,7 @@
         <v>25</v>
       </c>
       <c r="B30" s="25" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C30" s="26" t="n">
         <v>29</v>
@@ -14228,7 +13983,7 @@
         <v>25</v>
       </c>
       <c r="B31" s="25" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C31" s="26" t="n">
         <v>35</v>
@@ -14274,10 +14029,10 @@
         <v>21.1970491803279018</v>
       </c>
       <c r="R31" s="28" t="n">
-        <v>27.2093868255614915</v>
+        <v>27.2093868255614879</v>
       </c>
       <c r="S31" s="28" t="n">
-        <v>18.5746345520018927</v>
+        <v>18.5746345520018892</v>
       </c>
       <c r="T31" s="38">
         <f>S31-R31</f>
@@ -14289,7 +14044,7 @@
         <v>1000</v>
       </c>
       <c r="B32" s="25" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C32" s="26" t="n">
         <v>6</v>
@@ -14335,7 +14090,7 @@
         <v>11.0458074074074002</v>
       </c>
       <c r="R32" s="28" t="n">
-        <v>25.0831356048582919</v>
+        <v>25.0831356048582883</v>
       </c>
       <c r="S32" s="28" t="n">
         <v>15.8140211105345987</v>
@@ -14350,7 +14105,7 @@
         <v>1000</v>
       </c>
       <c r="B33" s="25" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="C33" s="26" t="n">
         <v>14</v>
@@ -14411,7 +14166,7 @@
         <v>1000</v>
       </c>
       <c r="B34" s="25" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C34" s="26" t="n">
         <v>22</v>
@@ -14457,7 +14212,7 @@
         <v>6.63054687500000028</v>
       </c>
       <c r="R34" s="28" t="n">
-        <v>18.2963008880614915</v>
+        <v>18.2963008880614879</v>
       </c>
       <c r="S34" s="28" t="n">
         <v>12.8405237197875</v>
@@ -14472,7 +14227,7 @@
         <v>1000</v>
       </c>
       <c r="B35" s="25" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C35" s="26" t="n">
         <v>30</v>
@@ -14511,7 +14266,7 @@
         <v>0.0379000000000000004</v>
       </c>
       <c r="P35" s="18" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="R35" s="28" t="n">
         <v>21.9923553466795987</v>
@@ -14529,7 +14284,7 @@
         <v>1000</v>
       </c>
       <c r="B36" s="25" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C36" s="26" t="n">
         <v>36</v>
@@ -14590,7 +14345,7 @@
         <v>1000</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C37" s="26" t="n">
         <v>45</v>
@@ -14651,7 +14406,7 @@
         <v>650</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C38" s="26" t="n">
         <v>7</v>
@@ -14712,7 +14467,7 @@
         <v>650</v>
       </c>
       <c r="B39" s="25" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C39" s="26" t="n">
         <v>15</v>
@@ -14773,7 +14528,7 @@
         <v>650</v>
       </c>
       <c r="B40" s="25" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C40" s="26" t="n">
         <v>23</v>
@@ -14834,7 +14589,7 @@
         <v>650</v>
       </c>
       <c r="B41" s="25" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C41" s="26" t="n">
         <v>46</v>
@@ -14895,7 +14650,7 @@
         <v>250</v>
       </c>
       <c r="B42" s="25" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="C42" s="26" t="n">
         <v>8</v>
@@ -14944,7 +14699,7 @@
         <v>17.205455780029201</v>
       </c>
       <c r="S42" s="28" t="n">
-        <v>13.4800510406494016</v>
+        <v>13.4800510406493999</v>
       </c>
       <c r="T42" s="38">
         <f>S42-R42</f>
@@ -14956,7 +14711,7 @@
         <v>250</v>
       </c>
       <c r="B43" s="25" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C43" s="26" t="n">
         <v>16</v>
@@ -15017,7 +14772,7 @@
         <v>250</v>
       </c>
       <c r="B44" s="25" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C44" s="26" t="n">
         <v>24</v>
@@ -15078,7 +14833,7 @@
         <v>250</v>
       </c>
       <c r="B45" s="25" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C45" s="26" t="n">
         <v>32</v>
@@ -15124,7 +14879,7 @@
         <v>3.93372990353697993</v>
       </c>
       <c r="R45" s="28" t="n">
-        <v>28.0284461975097017</v>
+        <v>28.0284461975096981</v>
       </c>
       <c r="S45" s="28" t="n">
         <v>16.9610939025877983</v>
@@ -15139,7 +14894,7 @@
         <v>250</v>
       </c>
       <c r="B46" s="25" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C46" s="26" t="n">
         <v>47</v>
@@ -15200,7 +14955,7 @@
         <v>100</v>
       </c>
       <c r="B47" s="25" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C47" s="26" t="n">
         <v>37</v>
@@ -15261,7 +15016,7 @@
         <v>100</v>
       </c>
       <c r="B48" s="25" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C48" s="26" t="n">
         <v>38</v>
@@ -15291,7 +15046,7 @@
         <v>0.0433218193138190077</v>
       </c>
       <c r="P48" s="18" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="R48" s="28" t="n">
         <v>21.5522689819335014</v>
@@ -15309,7 +15064,7 @@
         <v>100</v>
       </c>
       <c r="B49" s="25" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C49" s="26" t="n">
         <v>39</v>
@@ -15370,7 +15125,7 @@
         <v>100</v>
       </c>
       <c r="B50" s="25" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="C50" s="26" t="n">
         <v>40</v>
@@ -15416,7 +15171,7 @@
         <v>3.75387900355871995</v>
       </c>
       <c r="R50" s="28" t="n">
-        <v>19.7051658630370916</v>
+        <v>19.7051658630370881</v>
       </c>
       <c r="S50" s="28" t="n">
         <v>16.0419597625731996</v>
@@ -15431,7 +15186,7 @@
         <v>100</v>
       </c>
       <c r="B51" s="25" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C51" s="26" t="n">
         <v>48</v>
@@ -15477,7 +15232,7 @@
         <v>4.82783599088837967</v>
       </c>
       <c r="R51" s="28" t="n">
-        <v>18.720027923583892</v>
+        <v>18.7200279235838885</v>
       </c>
       <c r="S51" s="28" t="n">
         <v>14.3909511566162003</v>
@@ -15497,7 +15252,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1752044485" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1752046170" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -15506,14 +15261,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752044485" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752046170" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -15532,7 +15287,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="37" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -15596,10 +15351,10 @@
         <v>537</v>
       </c>
       <c r="C3" s="59" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D3" s="60" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E3" s="59" t="s">
         <v>80</v>
@@ -15675,7 +15430,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="60" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="E5" s="59" t="n">
         <v>19.8999999999999986</v>
@@ -15713,7 +15468,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="60" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E6" s="59" t="n">
         <v>20.6999999999999993</v>
@@ -15789,7 +15544,7 @@
         <v>5</v>
       </c>
       <c r="D8" s="60" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="E8" s="59" t="n">
         <v>9.40000000000000036</v>
@@ -15827,7 +15582,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="60" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E9" s="59" t="n">
         <v>20.3999999999999986</v>
@@ -15865,7 +15620,7 @@
         <v>7</v>
       </c>
       <c r="D10" s="60" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E10" s="59" t="n">
         <v>9.80000000000000071</v>
@@ -15941,7 +15696,7 @@
         <v>9</v>
       </c>
       <c r="D12" s="60" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E12" s="59" t="n">
         <v>11</v>
@@ -15979,7 +15734,7 @@
         <v>10</v>
       </c>
       <c r="D13" s="60" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E13" s="59" t="n">
         <v>19.6999999999999993</v>
@@ -16017,7 +15772,7 @@
         <v>11</v>
       </c>
       <c r="D14" s="60" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E14" s="59" t="n">
         <v>14.4000000000000004</v>
@@ -16055,7 +15810,7 @@
         <v>12</v>
       </c>
       <c r="D15" s="60" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="E15" s="59" t="n">
         <v>24.6000000000000014</v>
@@ -16093,7 +15848,7 @@
         <v>13</v>
       </c>
       <c r="D16" s="60" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="E16" s="59" t="n">
         <v>17.3000000000000007</v>
@@ -16131,7 +15886,7 @@
         <v>14</v>
       </c>
       <c r="D17" s="60" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E17" s="59" t="n">
         <v>11.0999999999999996</v>
@@ -16169,7 +15924,7 @@
         <v>15</v>
       </c>
       <c r="D18" s="60" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="E18" s="59" t="n">
         <v>21.5</v>
@@ -16207,7 +15962,7 @@
         <v>16</v>
       </c>
       <c r="D19" s="60" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="E19" s="59" t="n">
         <v>19.3999999999999986</v>
@@ -16245,7 +16000,7 @@
         <v>17</v>
       </c>
       <c r="D20" s="60" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E20" s="59" t="n">
         <v>13.9000000000000004</v>
@@ -16283,7 +16038,7 @@
         <v>18</v>
       </c>
       <c r="D21" s="60" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E21" s="59" t="n">
         <v>7</v>
@@ -16321,7 +16076,7 @@
         <v>19</v>
       </c>
       <c r="D22" s="60" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E22" s="59" t="n">
         <v>14.5</v>
@@ -16359,7 +16114,7 @@
         <v>20</v>
       </c>
       <c r="D23" s="60" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E23" s="59" t="n">
         <v>16.6000000000000014</v>
@@ -16397,7 +16152,7 @@
         <v>21</v>
       </c>
       <c r="D24" s="60" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="E24" s="59" t="n">
         <v>7.79999999999999982</v>
@@ -16435,7 +16190,7 @@
         <v>22</v>
       </c>
       <c r="D25" s="60" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E25" s="59" t="n">
         <v>9.5</v>
@@ -16473,7 +16228,7 @@
         <v>23</v>
       </c>
       <c r="D26" s="60" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E26" s="59" t="n">
         <v>22.3999999999999986</v>
@@ -16511,7 +16266,7 @@
         <v>24</v>
       </c>
       <c r="D27" s="60" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E27" s="59" t="n">
         <v>8.59999999999999787</v>
@@ -16549,7 +16304,7 @@
         <v>25</v>
       </c>
       <c r="D28" s="60" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E28" s="59" t="n">
         <v>18.1999999999999993</v>
@@ -16587,7 +16342,7 @@
         <v>26</v>
       </c>
       <c r="D29" s="60" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="E29" s="59" t="n">
         <v>12.5</v>
@@ -16625,7 +16380,7 @@
         <v>27</v>
       </c>
       <c r="D30" s="60" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E30" s="59" t="n">
         <v>11.5</v>
@@ -16663,7 +16418,7 @@
         <v>28</v>
       </c>
       <c r="D31" s="60" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E31" s="59" t="n">
         <v>7.90000000000000036</v>
@@ -16701,7 +16456,7 @@
         <v>29</v>
       </c>
       <c r="D32" s="60" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E32" s="59" t="n">
         <v>9.5</v>
@@ -16739,7 +16494,7 @@
         <v>30</v>
       </c>
       <c r="D33" s="60" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E33" s="59" t="n">
         <v>10.0999999999999996</v>
@@ -16777,7 +16532,7 @@
         <v>31</v>
       </c>
       <c r="D34" s="60" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E34" s="59" t="n">
         <v>21.5</v>
@@ -16815,7 +16570,7 @@
         <v>32</v>
       </c>
       <c r="D35" s="60" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E35" s="59" t="n">
         <v>19.8000000000000007</v>
@@ -16853,7 +16608,7 @@
         <v>33</v>
       </c>
       <c r="D36" s="60" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E36" s="59" t="n">
         <v>9.40000000000000036</v>
@@ -16891,7 +16646,7 @@
         <v>34</v>
       </c>
       <c r="D37" s="60" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E37" s="59" t="n">
         <v>9</v>
@@ -16929,7 +16684,7 @@
         <v>35</v>
       </c>
       <c r="D38" s="60" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E38" s="59" t="n">
         <v>18.5</v>
@@ -16967,7 +16722,7 @@
         <v>36</v>
       </c>
       <c r="D39" s="60" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E39" s="59" t="n">
         <v>14.6999999999999993</v>
@@ -17005,7 +16760,7 @@
         <v>37</v>
       </c>
       <c r="D40" s="60" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E40" s="59" t="n">
         <v>6.40000000000000036</v>
@@ -17043,7 +16798,7 @@
         <v>38</v>
       </c>
       <c r="D41" s="60" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E41" s="59" t="n">
         <v>7.90000000000000036</v>
@@ -17081,7 +16836,7 @@
         <v>39</v>
       </c>
       <c r="D42" s="60" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E42" s="59" t="n">
         <v>9.09999999999999964</v>
@@ -17119,7 +16874,7 @@
         <v>40</v>
       </c>
       <c r="D43" s="60" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E43" s="59" t="n">
         <v>20.3000000000000007</v>
@@ -17233,7 +16988,7 @@
         <v>43</v>
       </c>
       <c r="D46" s="60" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E46" s="59" t="n">
         <v>7.40000000000000036</v>
@@ -17271,7 +17026,7 @@
         <v>44</v>
       </c>
       <c r="D47" s="60" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E47" s="59" t="n">
         <v>6.59999999999999964</v>
@@ -17309,7 +17064,7 @@
         <v>45</v>
       </c>
       <c r="D48" s="60" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="E48" s="59" t="n">
         <v>10.0999999999999996</v>
@@ -17385,7 +17140,7 @@
         <v>47</v>
       </c>
       <c r="D50" s="60" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E50" s="59" t="n">
         <v>9.09999999999999964</v>
@@ -17423,7 +17178,7 @@
         <v>48</v>
       </c>
       <c r="D51" s="60" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="E51" s="59" t="n">
         <v>20.3000000000000007</v>
@@ -17461,7 +17216,7 @@
         <v>49</v>
       </c>
       <c r="D52" s="60" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E52" s="59" t="n">
         <v>10.5999999999999996</v>
@@ -17499,7 +17254,7 @@
         <v>50</v>
       </c>
       <c r="D53" s="60" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="E53" s="59" t="n">
         <v>6.09999999999999964</v>
@@ -17537,7 +17292,7 @@
         <v>51</v>
       </c>
       <c r="D54" s="60" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E54" s="59" t="n">
         <v>16.6000000000000014</v>
@@ -17575,7 +17330,7 @@
         <v>52</v>
       </c>
       <c r="D55" s="60" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="E55" s="59" t="n">
         <v>16.1999999999999993</v>
@@ -17613,7 +17368,7 @@
         <v>53</v>
       </c>
       <c r="D56" s="60" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="E56" s="59" t="n">
         <v>15.4000000000000004</v>
@@ -17651,7 +17406,7 @@
         <v>54</v>
       </c>
       <c r="D57" s="60" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E57" s="59" t="n">
         <v>7</v>
@@ -17689,7 +17444,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="60" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="E58" s="59" t="n">
         <v>18</v>
@@ -17727,7 +17482,7 @@
         <v>2</v>
       </c>
       <c r="D59" s="60" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E59" s="59" t="n">
         <v>16.1999999999999993</v>
@@ -17765,7 +17520,7 @@
         <v>3</v>
       </c>
       <c r="D60" s="60" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="E60" s="59" t="n">
         <v>21.3000000000000007</v>
@@ -17803,7 +17558,7 @@
         <v>4</v>
       </c>
       <c r="D61" s="60" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E61" s="59" t="n">
         <v>21.1000000000000014</v>
@@ -17841,7 +17596,7 @@
         <v>5</v>
       </c>
       <c r="D62" s="60" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="E62" s="59" t="n">
         <v>19.1000000000000014</v>
@@ -17879,7 +17634,7 @@
         <v>6</v>
       </c>
       <c r="D63" s="60" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E63" s="59" t="n">
         <v>12.5</v>
@@ -17917,7 +17672,7 @@
         <v>7</v>
       </c>
       <c r="D64" s="60" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E64" s="59" t="n">
         <v>21.3999999999999986</v>
@@ -17955,7 +17710,7 @@
         <v>8</v>
       </c>
       <c r="D65" s="60" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E65" s="59" t="n">
         <v>18.1999999999999993</v>
@@ -17993,7 +17748,7 @@
         <v>9</v>
       </c>
       <c r="D66" s="60" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="E66" s="59" t="n">
         <v>20.6000000000000014</v>
@@ -18031,7 +17786,7 @@
         <v>10</v>
       </c>
       <c r="D67" s="60" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="E67" s="59" t="n">
         <v>19.3000000000000007</v>
@@ -18069,7 +17824,7 @@
         <v>11</v>
       </c>
       <c r="D68" s="60" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="E68" s="59" t="n">
         <v>18.8000000000000007</v>
@@ -18107,7 +17862,7 @@
         <v>12</v>
       </c>
       <c r="D69" s="60" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E69" s="59" t="n">
         <v>12.1999999999999993</v>
@@ -18145,7 +17900,7 @@
         <v>13</v>
       </c>
       <c r="D70" s="60" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="E70" s="59" t="n">
         <v>14.4000000000000004</v>
@@ -18183,7 +17938,7 @@
         <v>14</v>
       </c>
       <c r="D71" s="60" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="E71" s="59" t="n">
         <v>18.1000000000000014</v>
@@ -18221,7 +17976,7 @@
         <v>15</v>
       </c>
       <c r="D72" s="60" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="E72" s="59" t="n">
         <v>17.1999999999999993</v>
@@ -18259,7 +18014,7 @@
         <v>16</v>
       </c>
       <c r="D73" s="60" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E73" s="59" t="n">
         <v>14.1999999999999993</v>
@@ -18297,7 +18052,7 @@
         <v>17</v>
       </c>
       <c r="D74" s="60" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E74" s="59" t="n">
         <v>18.1000000000000014</v>
@@ -18335,7 +18090,7 @@
         <v>18</v>
       </c>
       <c r="D75" s="60" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="E75" s="59" t="n">
         <v>18.5</v>
@@ -18373,7 +18128,7 @@
         <v>19</v>
       </c>
       <c r="D76" s="60" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="E76" s="59" t="n">
         <v>19.3000000000000007</v>
@@ -18411,7 +18166,7 @@
         <v>1</v>
       </c>
       <c r="D77" s="60" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="E77" s="59" t="n">
         <v>27.1999999999999993</v>
@@ -18449,7 +18204,7 @@
         <v>2</v>
       </c>
       <c r="D78" s="60" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E78" s="59" t="n">
         <v>18.6000000000000014</v>
@@ -18487,7 +18242,7 @@
         <v>3</v>
       </c>
       <c r="D79" s="60" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="E79" s="59" t="n">
         <v>25.8000000000000007</v>
@@ -18525,7 +18280,7 @@
         <v>4</v>
       </c>
       <c r="D80" s="60" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="E80" s="59" t="n">
         <v>29.3999999999999986</v>
@@ -18563,7 +18318,7 @@
         <v>5</v>
       </c>
       <c r="D81" s="60" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="E81" s="59" t="n">
         <v>24.1999999999999993</v>
@@ -18601,7 +18356,7 @@
         <v>6</v>
       </c>
       <c r="D82" s="60" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E82" s="59" t="n">
         <v>11.4000000000000004</v>
@@ -18639,7 +18394,7 @@
         <v>7</v>
       </c>
       <c r="D83" s="60" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="E83" s="59" t="n">
         <v>20</v>
@@ -18677,7 +18432,7 @@
         <v>8</v>
       </c>
       <c r="D84" s="60" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="E84" s="59" t="n">
         <v>25.3999999999999986</v>
@@ -18715,7 +18470,7 @@
         <v>9</v>
       </c>
       <c r="D85" s="60" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="E85" s="59" t="n">
         <v>16.1000000000000014</v>
@@ -18753,7 +18508,7 @@
         <v>10</v>
       </c>
       <c r="D86" s="60" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E86" s="59" t="n">
         <v>14.6999999999999993</v>
@@ -18791,7 +18546,7 @@
         <v>11</v>
       </c>
       <c r="D87" s="60" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="E87" s="59" t="n">
         <v>19.6999999999999993</v>
@@ -18829,7 +18584,7 @@
         <v>12</v>
       </c>
       <c r="D88" s="60" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="E88" s="59" t="n">
         <v>8.59999999999999787</v>
@@ -18867,7 +18622,7 @@
         <v>13</v>
       </c>
       <c r="D89" s="60" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E89" s="59" t="n">
         <v>11.1999999999999993</v>
@@ -18905,7 +18660,7 @@
         <v>14</v>
       </c>
       <c r="D90" s="60" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="E90" s="59" t="n">
         <v>17.399999999999995</v>
@@ -18943,7 +18698,7 @@
         <v>15</v>
       </c>
       <c r="D91" s="60" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E91" s="59" t="n">
         <v>19.1999999999999993</v>
@@ -18981,7 +18736,7 @@
         <v>16</v>
       </c>
       <c r="D92" s="60" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="E92" s="59" t="n">
         <v>26.5</v>
@@ -19019,7 +18774,7 @@
         <v>1</v>
       </c>
       <c r="D93" s="60" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="E93" s="59" t="n">
         <v>18.1000000000000014</v>
@@ -19057,7 +18812,7 @@
         <v>2</v>
       </c>
       <c r="D94" s="60" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E94" s="59" t="n">
         <v>21.3000000000000007</v>
@@ -19095,7 +18850,7 @@
         <v>3</v>
       </c>
       <c r="D95" s="60" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="E95" s="59" t="n">
         <v>19.3000000000000007</v>
@@ -19133,7 +18888,7 @@
         <v>4</v>
       </c>
       <c r="D96" s="60" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E96" s="59" t="n">
         <v>24.6999999999999993</v>
@@ -19171,7 +18926,7 @@
         <v>5</v>
       </c>
       <c r="D97" s="60" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="E97" s="59" t="n">
         <v>22.3999999999999986</v>
@@ -19209,7 +18964,7 @@
         <v>6</v>
       </c>
       <c r="D98" s="60" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E98" s="59" t="n">
         <v>18.3999999999999986</v>
@@ -19247,7 +19002,7 @@
         <v>7</v>
       </c>
       <c r="D99" s="60" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="E99" s="59" t="n">
         <v>19.5</v>
@@ -19285,7 +19040,7 @@
         <v>8</v>
       </c>
       <c r="D100" s="60" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="E100" s="59" t="n">
         <v>23.5</v>
@@ -19323,7 +19078,7 @@
         <v>9</v>
       </c>
       <c r="D101" s="60" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E101" s="59" t="n">
         <v>25.1000000000000014</v>
@@ -19361,7 +19116,7 @@
         <v>10</v>
       </c>
       <c r="D102" s="60" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="E102" s="59" t="n">
         <v>28.6000000000000014</v>
@@ -19399,7 +19154,7 @@
         <v>11</v>
       </c>
       <c r="D103" s="60" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="E103" s="59" t="n">
         <v>28.6999999999999993</v>
@@ -19437,7 +19192,7 @@
         <v>12</v>
       </c>
       <c r="D104" s="60" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="E104" s="59" t="n">
         <v>23.6000000000000014</v>
@@ -19475,7 +19230,7 @@
         <v>13</v>
       </c>
       <c r="D105" s="60" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E105" s="59" t="n">
         <v>21.8000000000000007</v>
@@ -19513,7 +19268,7 @@
         <v>14</v>
       </c>
       <c r="D106" s="60" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="E106" s="59" t="n">
         <v>25.1999999999999993</v>
@@ -19551,7 +19306,7 @@
         <v>15</v>
       </c>
       <c r="D107" s="60" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="E107" s="59" t="n">
         <v>22.1000000000000014</v>
@@ -19589,7 +19344,7 @@
         <v>16</v>
       </c>
       <c r="D108" s="60" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="E108" s="59" t="n">
         <v>24.1999999999999993</v>
@@ -19627,7 +19382,7 @@
         <v>17</v>
       </c>
       <c r="D109" s="60" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E109" s="59" t="n">
         <v>22.3999999999999986</v>
@@ -19665,7 +19420,7 @@
         <v>18</v>
       </c>
       <c r="D110" s="60" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="E110" s="59" t="n">
         <v>26.5</v>
@@ -19703,7 +19458,7 @@
         <v>19</v>
       </c>
       <c r="D111" s="60" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E111" s="59" t="n">
         <v>25.1000000000000014</v>
@@ -19741,7 +19496,7 @@
         <v>20</v>
       </c>
       <c r="D112" s="60" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E112" s="59" t="n">
         <v>24.1000000000000014</v>
@@ -19779,7 +19534,7 @@
         <v>21</v>
       </c>
       <c r="D113" s="60" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E113" s="59" t="n">
         <v>20.6999999999999993</v>
@@ -19817,7 +19572,7 @@
         <v>22</v>
       </c>
       <c r="D114" s="60" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="E114" s="59" t="n">
         <v>19.6000000000000014</v>
@@ -19855,7 +19610,7 @@
         <v>23</v>
       </c>
       <c r="D115" s="60" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="E115" s="59" t="n">
         <v>24.6999999999999993</v>
@@ -19893,7 +19648,7 @@
         <v>24</v>
       </c>
       <c r="D116" s="60" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="E116" s="59" t="n">
         <v>12.1999999999999993</v>
@@ -19931,7 +19686,7 @@
         <v>1</v>
       </c>
       <c r="D117" s="60" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="E117" s="59" t="n">
         <v>21.1000000000000014</v>
@@ -19969,7 +19724,7 @@
         <v>2</v>
       </c>
       <c r="D118" s="60" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="E118" s="59" t="n">
         <v>20.3000000000000007</v>
@@ -20007,7 +19762,7 @@
         <v>3</v>
       </c>
       <c r="D119" s="60" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="E119" s="59" t="n">
         <v>21.3000000000000007</v>
@@ -20045,7 +19800,7 @@
         <v>4</v>
       </c>
       <c r="D120" s="60" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="E120" s="59" t="n">
         <v>25.1999999999999993</v>
@@ -20083,7 +19838,7 @@
         <v>5</v>
       </c>
       <c r="D121" s="60" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="E121" s="59" t="n">
         <v>18</v>
@@ -20121,7 +19876,7 @@
         <v>6</v>
       </c>
       <c r="D122" s="60" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E122" s="59" t="n">
         <v>22.8000000000000007</v>
@@ -20159,7 +19914,7 @@
         <v>7</v>
       </c>
       <c r="D123" s="60" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="E123" s="59" t="n">
         <v>23.1000000000000014</v>
@@ -20197,7 +19952,7 @@
         <v>8</v>
       </c>
       <c r="D124" s="60" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="E124" s="59" t="n">
         <v>15.5</v>
@@ -20235,7 +19990,7 @@
         <v>9</v>
       </c>
       <c r="D125" s="60" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="E125" s="59" t="n">
         <v>23.8999999999999986</v>
@@ -20273,7 +20028,7 @@
         <v>10</v>
       </c>
       <c r="D126" s="60" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E126" s="59" t="n">
         <v>22.8000000000000007</v>
@@ -20311,7 +20066,7 @@
         <v>11</v>
       </c>
       <c r="D127" s="60" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E127" s="59" t="n">
         <v>23.1999999999999993</v>
@@ -20349,7 +20104,7 @@
         <v>12</v>
       </c>
       <c r="D128" s="60" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="E128" s="59" t="n">
         <v>18</v>
@@ -20387,7 +20142,7 @@
         <v>13</v>
       </c>
       <c r="D129" s="60" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E129" s="59" t="n">
         <v>22</v>
@@ -20425,7 +20180,7 @@
         <v>14</v>
       </c>
       <c r="D130" s="60" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E130" s="59" t="n">
         <v>23.6999999999999993</v>
@@ -20463,7 +20218,7 @@
         <v>15</v>
       </c>
       <c r="D131" s="60" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="E131" s="59" t="n">
         <v>23</v>
@@ -20501,7 +20256,7 @@
         <v>16</v>
       </c>
       <c r="D132" s="60" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="E132" s="59" t="n">
         <v>23.8000000000000007</v>
@@ -20539,7 +20294,7 @@
         <v>17</v>
       </c>
       <c r="D133" s="60" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="E133" s="59" t="n">
         <v>21</v>
@@ -20577,7 +20332,7 @@
         <v>18</v>
       </c>
       <c r="D134" s="60" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="E134" s="59" t="n">
         <v>23.1000000000000014</v>
@@ -20615,7 +20370,7 @@
         <v>19</v>
       </c>
       <c r="D135" s="60" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E135" s="59" t="n">
         <v>26.3999999999999986</v>
@@ -20653,7 +20408,7 @@
         <v>20</v>
       </c>
       <c r="D136" s="60" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E136" s="59" t="n">
         <v>23.8999999999999986</v>
@@ -20691,7 +20446,7 @@
         <v>21</v>
       </c>
       <c r="D137" s="60" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E137" s="59" t="n">
         <v>23.8000000000000007</v>
@@ -20729,7 +20484,7 @@
         <v>22</v>
       </c>
       <c r="D138" s="60" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="E138" s="59" t="n">
         <v>26.3000000000000007</v>
@@ -20767,7 +20522,7 @@
         <v>23</v>
       </c>
       <c r="D139" s="60" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="E139" s="59" t="n">
         <v>20.1000000000000014</v>
@@ -20805,7 +20560,7 @@
         <v>24</v>
       </c>
       <c r="D140" s="60" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="E140" s="59" t="n">
         <v>28.8999999999999986</v>
@@ -20843,7 +20598,7 @@
         <v>25</v>
       </c>
       <c r="D141" s="60" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="E141" s="59" t="n">
         <v>16.5</v>
@@ -20881,7 +20636,7 @@
         <v>26</v>
       </c>
       <c r="D142" s="60" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="E142" s="59" t="n">
         <v>21.8000000000000007</v>
@@ -20919,7 +20674,7 @@
         <v>27</v>
       </c>
       <c r="D143" s="60" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="E143" s="59" t="n">
         <v>17.1000000000000014</v>
@@ -20957,7 +20712,7 @@
         <v>28</v>
       </c>
       <c r="D144" s="60" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="E144" s="59" t="n">
         <v>16.5</v>
@@ -20995,7 +20750,7 @@
         <v>29</v>
       </c>
       <c r="D145" s="60" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E145" s="59" t="n">
         <v>19.8000000000000007</v>
@@ -44994,7 +44749,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1752044485" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1752046170" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -45003,14 +44758,14 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1752044485" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:header xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1752046170" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752044485" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1752046170" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>